<commit_message>
requiements updated, follow ProductBacklog_2.xlsx
</commit_message>
<xml_diff>
--- a/Docs/ProductBacklog_2.xlsx
+++ b/Docs/ProductBacklog_2.xlsx
@@ -255,7 +255,7 @@
     <t xml:space="preserve">Skip &amp; Like</t>
   </si>
   <si>
-    <t xml:space="preserve">Skip to next song or like/dislike track</t>
+    <t xml:space="preserve">Skip to next song or like/dislike track (these happen in RedDust, not music streaming app)</t>
   </si>
   <si>
     <t xml:space="preserve">Personal Memory System</t>
@@ -582,7 +582,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -607,58 +607,42 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -675,28 +659,16 @@
       <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1257,24 +1229,24 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="55"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="6" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="51.47"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="1" width="10.16"/>
   </cols>
   <sheetData>
-    <row r="1" s="10" customFormat="true" ht="30.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+    <row r="1" s="3" customFormat="true" ht="30.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="9" t="s">
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1282,16 +1254,16 @@
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2" s="11" t="s">
+      <c r="B2" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="10" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1300,13 +1272,13 @@
       <c r="B3" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="12" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1315,324 +1287,324 @@
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="16" t="s">
+      <c r="C4" s="8"/>
+      <c r="D4" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="14" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="16" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="21" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="18" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="23" t="s">
+      <c r="C7" s="8"/>
+      <c r="D7" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="14" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="12" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="23" t="s">
+      <c r="C9" s="8"/>
+      <c r="D9" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="14" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="26" t="s">
+      <c r="E10" s="12" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="27" t="s">
+      <c r="C11" s="8"/>
+      <c r="D11" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="E11" s="28" t="s">
+      <c r="E11" s="20" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="23" t="s">
+      <c r="C12" s="8"/>
+      <c r="D12" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="14" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="D13" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E13" s="26" t="s">
+      <c r="E13" s="12" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="27" t="s">
+      <c r="C14" s="8"/>
+      <c r="D14" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="E14" s="28" t="s">
+      <c r="E14" s="20" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="30.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="23" t="s">
+      <c r="C15" s="8"/>
+      <c r="D15" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="E15" s="24" t="s">
+      <c r="E15" s="21" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="D16" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="12" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5"/>
       <c r="B17" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="27" t="s">
+      <c r="C17" s="8"/>
+      <c r="D17" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="E17" s="28" t="s">
+      <c r="E17" s="20" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5"/>
       <c r="B18" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C18" s="18"/>
-      <c r="D18" s="27" t="s">
+      <c r="C18" s="8"/>
+      <c r="D18" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="20" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5"/>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="18"/>
-      <c r="D19" s="23" t="s">
+      <c r="C19" s="8"/>
+      <c r="D19" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="E19" s="14" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5"/>
       <c r="B20" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D20" s="25" t="s">
+      <c r="D20" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="E20" s="26" t="s">
+      <c r="E20" s="12" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5"/>
       <c r="B21" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="27" t="s">
+      <c r="C21" s="8"/>
+      <c r="D21" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="E21" s="28" t="s">
+      <c r="E21" s="20" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5"/>
       <c r="B22" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C22" s="18"/>
-      <c r="D22" s="27" t="s">
+      <c r="C22" s="8"/>
+      <c r="D22" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="E22" s="28" t="s">
+      <c r="E22" s="20" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5"/>
       <c r="B23" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C23" s="18"/>
-      <c r="D23" s="23" t="s">
+      <c r="C23" s="8"/>
+      <c r="D23" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="14" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5"/>
       <c r="B24" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="D24" s="25" t="s">
+      <c r="D24" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="E24" s="26" t="s">
+      <c r="E24" s="12" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5"/>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C25" s="18"/>
-      <c r="D25" s="27" t="s">
+      <c r="C25" s="8"/>
+      <c r="D25" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="E25" s="28" t="s">
+      <c r="E25" s="20" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5"/>
       <c r="B26" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C26" s="18"/>
-      <c r="D26" s="27" t="s">
+      <c r="C26" s="8"/>
+      <c r="D26" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="E26" s="28" t="s">
+      <c r="E26" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5"/>
       <c r="B27" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C27" s="18"/>
-      <c r="D27" s="27" t="s">
+      <c r="C27" s="8"/>
+      <c r="D27" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="E27" s="28" t="s">
+      <c r="E27" s="20" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1641,11 +1613,11 @@
       <c r="B28" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="27" t="s">
+      <c r="C28" s="8"/>
+      <c r="D28" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="E28" s="28" t="s">
+      <c r="E28" s="20" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1654,11 +1626,11 @@
       <c r="B29" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C29" s="18"/>
-      <c r="D29" s="23" t="s">
+      <c r="C29" s="8"/>
+      <c r="D29" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="E29" s="24" t="s">
+      <c r="E29" s="14" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1667,13 +1639,13 @@
       <c r="B30" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D30" s="25" t="s">
+      <c r="D30" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="E30" s="26" t="s">
+      <c r="E30" s="12" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1682,11 +1654,11 @@
       <c r="B31" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C31" s="18"/>
-      <c r="D31" s="27" t="s">
+      <c r="C31" s="8"/>
+      <c r="D31" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="E31" s="28" t="s">
+      <c r="E31" s="20" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1695,11 +1667,11 @@
       <c r="B32" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C32" s="18"/>
-      <c r="D32" s="23" t="s">
+      <c r="C32" s="8"/>
+      <c r="D32" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="E32" s="24" t="s">
+      <c r="E32" s="14" t="s">
         <v>115</v>
       </c>
     </row>
@@ -1708,13 +1680,13 @@
       <c r="B33" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C33" s="18" t="s">
+      <c r="C33" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="D33" s="25" t="s">
+      <c r="D33" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="E33" s="26" t="s">
+      <c r="E33" s="12" t="s">
         <v>118</v>
       </c>
     </row>
@@ -1723,11 +1695,11 @@
       <c r="B34" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C34" s="18"/>
-      <c r="D34" s="27" t="s">
+      <c r="C34" s="8"/>
+      <c r="D34" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E34" s="28" t="s">
+      <c r="E34" s="20" t="s">
         <v>120</v>
       </c>
     </row>
@@ -1736,11 +1708,11 @@
       <c r="B35" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C35" s="18"/>
-      <c r="D35" s="23" t="s">
+      <c r="C35" s="8"/>
+      <c r="D35" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="E35" s="24" t="s">
+      <c r="E35" s="14" t="s">
         <v>122</v>
       </c>
     </row>
@@ -1776,71 +1748,71 @@
   <dimension ref="A1:A13"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="29" width="73.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="22" width="73.31"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="22" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="22" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="22" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="22" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="22" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="22" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="22" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="22" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="22" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="22" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="22" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="22" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29" t="s">
+      <c r="A13" s="22" t="s">
         <v>135</v>
       </c>
     </row>

</xml_diff>